<commit_message>
fix: lme integrity fix + data upload
</commit_message>
<xml_diff>
--- a/LME/parser/antimony/data/antimony.xlsx
+++ b/LME/parser/antimony/data/antimony.xlsx
@@ -28,7 +28,7 @@
     <t>104500</t>
   </si>
   <si>
-    <t>13728.7</t>
+    <t>13726.66</t>
   </si>
 </sst>
 </file>
@@ -390,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C616"/>
+  <dimension ref="A1:C617"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -7159,10 +7159,21 @@
       <c r="A616" s="2">
         <v>46266</v>
       </c>
-      <c r="B616" t="s">
+      <c r="B616">
+        <v>104500</v>
+      </c>
+      <c r="C616">
+        <v>13728.7</v>
+      </c>
+    </row>
+    <row r="617" spans="1:3">
+      <c r="A617" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B617" t="s">
         <v>3</v>
       </c>
-      <c r="C616" t="s">
+      <c r="C617" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>